<commit_message>
Přidána nová závada ID 775 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I710"/>
+  <dimension ref="A1:I711"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24128,6 +24128,43 @@
         </is>
       </c>
     </row>
+    <row r="711">
+      <c r="A711" t="n">
+        <v>775</v>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>15.09.2026</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>Za jízdy občas nasvítí N2, vyměnili pouze snímač směrového válce mechaniku nechali</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr"/>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G711" t="inlineStr"/>
+      <c r="H711" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I711" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 776 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I711"/>
+  <dimension ref="A1:I712"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24165,6 +24165,47 @@
         </is>
       </c>
     </row>
+    <row r="712">
+      <c r="A712" t="n">
+        <v>776</v>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>16.09.2026</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>Nedobíjí B, podle kódu blikající LED přehřátí generátoru (otrokovice)</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>v depu oprava konektoru pod velkým deklem generátoru C1-C2 měli 125 Ohm</t>
+        </is>
+      </c>
+      <c r="F712" t="inlineStr">
+        <is>
+          <t>Dobíjení</t>
+        </is>
+      </c>
+      <c r="G712" t="inlineStr"/>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I712" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 777 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I712"/>
+  <dimension ref="A1:I713"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24206,6 +24206,43 @@
         </is>
       </c>
     </row>
+    <row r="713">
+      <c r="A713" t="n">
+        <v>777</v>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>20.09.2026</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>Červený alarm motoru B v SAMu hlásí alarm teploty vyšší jak 105 stupňů ,motorari vyměnili chladič a termostat</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr"/>
+      <c r="F713" t="inlineStr">
+        <is>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G713" t="inlineStr"/>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I713" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 778 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I713"/>
+  <dimension ref="A1:I714"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24243,6 +24243,43 @@
         </is>
       </c>
     </row>
+    <row r="714">
+      <c r="A714" t="n">
+        <v>778</v>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>844 014</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>16.09.2026</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>Bez komunikace CPU1, firovi stopovala mašina ,výměna  zdrojovky a CPU1</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr"/>
+      <c r="F714" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G714" t="inlineStr"/>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I714" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 779 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I714"/>
+  <dimension ref="A1:I715"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24280,6 +24280,43 @@
         </is>
       </c>
     </row>
+    <row r="715">
+      <c r="A715" t="n">
+        <v>779</v>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>844 025</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>22.09.2026</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>Výměna jízdní páky na B , nešla potvrdit do výkonu</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr"/>
+      <c r="F715" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G715" t="inlineStr"/>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 780 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I715"/>
+  <dimension ref="A1:I716"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24317,6 +24317,43 @@
         </is>
       </c>
     </row>
+    <row r="716">
+      <c r="A716" t="n">
+        <v>780</v>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>16.09.2026</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>Vadný požární kabel na motoru B, upadl chladič taky na B - oprava konektoru pro zobrazovače AD-Blue</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr"/>
+      <c r="F716" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G716" t="inlineStr"/>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I716" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 781 (autor: Petr)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I716"/>
+  <dimension ref="A1:I717"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24354,6 +24354,47 @@
         </is>
       </c>
     </row>
+    <row r="717">
+      <c r="A717" t="n">
+        <v>781</v>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>04.10.2026</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>Vadny pozarni kabel na B motore. Vymena za  novy.</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>Pouzilibjsme je 13,5 m</t>
+        </is>
+      </c>
+      <c r="F717" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G717" t="inlineStr"/>
+      <c r="H717" t="inlineStr">
+        <is>
+          <t>Petr</t>
+        </is>
+      </c>
+      <c r="I717" t="inlineStr">
+        <is>
+          <t>Petr</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 782 (autor: Petr)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I717"/>
+  <dimension ref="A1:I718"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24395,6 +24395,47 @@
         </is>
       </c>
     </row>
+    <row r="718">
+      <c r="A718" t="n">
+        <v>782</v>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>04.10.2026</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>Vadny pozarni kabel na B motore. Vymena za  novy.</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>Pouzilibjsme je 13,5 m</t>
+        </is>
+      </c>
+      <c r="F718" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G718" t="inlineStr"/>
+      <c r="H718" t="inlineStr">
+        <is>
+          <t>Petr</t>
+        </is>
+      </c>
+      <c r="I718" t="inlineStr">
+        <is>
+          <t>Petr</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Smazána závada ID 782 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I718"/>
+  <dimension ref="A1:I717"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24395,47 +24395,6 @@
         </is>
       </c>
     </row>
-    <row r="718">
-      <c r="A718" t="n">
-        <v>782</v>
-      </c>
-      <c r="B718" t="inlineStr">
-        <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C718" t="inlineStr">
-        <is>
-          <t>04.10.2026</t>
-        </is>
-      </c>
-      <c r="D718" t="inlineStr">
-        <is>
-          <t>Vadny pozarni kabel na B motore. Vymena za  novy.</t>
-        </is>
-      </c>
-      <c r="E718" t="inlineStr">
-        <is>
-          <t>Pouzilibjsme je 13,5 m</t>
-        </is>
-      </c>
-      <c r="F718" t="inlineStr">
-        <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G718" t="inlineStr"/>
-      <c r="H718" t="inlineStr">
-        <is>
-          <t>Petr</t>
-        </is>
-      </c>
-      <c r="I718" t="inlineStr">
-        <is>
-          <t>Petr</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 782 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I717"/>
+  <dimension ref="A1:I718"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24395,6 +24395,43 @@
         </is>
       </c>
     </row>
+    <row r="718">
+      <c r="A718" t="n">
+        <v>782</v>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>05.10.2026</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>Výměna náhonu ETCS 2 osa č.1</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr"/>
+      <c r="F718" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G718" t="inlineStr"/>
+      <c r="H718" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I718" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 783 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I718"/>
+  <dimension ref="A1:I719"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24432,6 +24432,47 @@
         </is>
       </c>
     </row>
+    <row r="719">
+      <c r="A719" t="n">
+        <v>783</v>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>814 063</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>08.10.2026</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>Výměna displeje Lokel na 814</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>Použity z 814 028 po vyhoření</t>
+        </is>
+      </c>
+      <c r="F719" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G719" t="inlineStr"/>
+      <c r="H719" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I719" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 784 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I719"/>
+  <dimension ref="A1:I720"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24473,6 +24473,47 @@
         </is>
       </c>
     </row>
+    <row r="720">
+      <c r="A720" t="n">
+        <v>784</v>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>Na A levé dveře při zavření dveří stále svítí tlačitka otevření a osvětlení nástupního protoru, zjištěn zkrat mezi vodiči 810 a 824, nad dveřma je odpojený vodič 824</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>Chtělo by to až bude odstavena projít ještě výdejní okno jestli to tam není někde propojené</t>
+        </is>
+      </c>
+      <c r="F720" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G720" t="inlineStr"/>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 785 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I720"/>
+  <dimension ref="A1:I721"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24514,6 +24514,43 @@
         </is>
       </c>
     </row>
+    <row r="721">
+      <c r="A721" t="n">
+        <v>785</v>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>Při snížení slaku o 1 bar se nasvítí kontrolka plnění 5 barů, zjištěn rozepnutý prostřední podvozek SP18.2 - výměna</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr"/>
+      <c r="F721" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G721" t="inlineStr"/>
+      <c r="H721" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 786 (autor: Petr)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I721"/>
+  <dimension ref="A1:I722"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24551,6 +24551,43 @@
         </is>
       </c>
     </row>
+    <row r="722">
+      <c r="A722" t="n">
+        <v>786</v>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>842 010</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>23.10.2026</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>Nejde odvetravani ETCS skrine. Provizorne dosazen ventilator s mensim vykonem. Az se tu ukaze vymenit na original</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr"/>
+      <c r="F722" t="inlineStr">
+        <is>
+          <t>VZ - Radiostanice</t>
+        </is>
+      </c>
+      <c r="G722" t="inlineStr"/>
+      <c r="H722" t="inlineStr">
+        <is>
+          <t>Petr</t>
+        </is>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>Petr</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 787 (autor: Dan)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I722"/>
+  <dimension ref="A1:I723"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24588,6 +24588,47 @@
         </is>
       </c>
     </row>
+    <row r="723">
+      <c r="A723" t="n">
+        <v>787</v>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>26.10.2026</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>Vypadává směr na A</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>Prověření linky od směrového válce do konektoru SAM- OK -&gt; přehození SAMů mezi sebou (A&lt;-&gt;B)</t>
+        </is>
+      </c>
+      <c r="F723" t="inlineStr">
+        <is>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G723" t="inlineStr"/>
+      <c r="H723" t="inlineStr">
+        <is>
+          <t>Dan</t>
+        </is>
+      </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>Dan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 788 (autor: Dan)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I723"/>
+  <dimension ref="A1:I724"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24629,6 +24629,47 @@
         </is>
       </c>
     </row>
+    <row r="724">
+      <c r="A724" t="n">
+        <v>788</v>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>814 002</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>26.10.2026</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>Opakovaně se samovolně restartuje, jedna nebo druhá půlka infosystému.</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>IS se nerozpadl - nedelano (za mě OK)</t>
+        </is>
+      </c>
+      <c r="F724" t="inlineStr">
+        <is>
+          <t>IS - Infosystém</t>
+        </is>
+      </c>
+      <c r="G724" t="inlineStr"/>
+      <c r="H724" t="inlineStr">
+        <is>
+          <t>Dan</t>
+        </is>
+      </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>Dan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hromadná úprava z tabulky (Radek) (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -26749,11 +26749,11 @@
       </c>
       <c r="I722" t="inlineStr">
         <is>
-          <t>Petr</t>
+          <t>Radek</t>
         </is>
       </c>
       <c r="J722" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="723">

</xml_diff>